<commit_message>
Add Cantonese (yue) dialect support with ToJyutping
Co-authored-by: indiejoseph <577551+indiejoseph@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dialect_frontend/frontend/dialect/yue/tone.xlsx
+++ b/dialect_frontend/frontend/dialect/yue/tone.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ᴴᴴ</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -455,7 +455,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ᴹᴴ</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -467,7 +467,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ᴹᴹ</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -479,7 +479,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ᴸᴹ</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ᴸᴴ</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -503,7 +503,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ᴸᴸ</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>